<commit_message>
feat: evaluated 3 new LSTM architectures and renamed evaluation script
</commit_message>
<xml_diff>
--- a/data/experiment_logs.xlsx
+++ b/data/experiment_logs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saadm\Documents\gridops-ai\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00FA59BD-2C9E-417D-8017-E3C4F9840B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62B8A190-E425-4C2C-94C7-106D0BB97E84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="41">
   <si>
     <t>experiment_id</t>
   </si>
@@ -132,12 +132,42 @@
   </si>
   <si>
     <t>activation_function</t>
+  </si>
+  <si>
+    <t>lstm_4</t>
+  </si>
+  <si>
+    <t>lstm_5</t>
+  </si>
+  <si>
+    <t>lstm_6</t>
+  </si>
+  <si>
+    <t>Lower validation loss with Huber loss, but evaluation metrics show higher overall error and reduced R2</t>
+  </si>
+  <si>
+    <t>Not selected; compare loss metric performance against MSE-trained models</t>
+  </si>
+  <si>
+    <t>Premature early stopping resulted in underfitting, leading to poor R2 variance score and higher forecast error</t>
+  </si>
+  <si>
+    <t>Not selected; adjust patience or learning rate schedule to allow sufficient convergence</t>
+  </si>
+  <si>
+    <t>Loss curves show mild fluctuations with validation loss stabilising around 0.08, the actual vs. predicted plot shows consistent underprediction on high-demand peaks</t>
+  </si>
+  <si>
+    <t>Not selected; short lookback fails to capture long-term seasonal peaks adequately</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -173,7 +203,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -181,43 +211,54 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="19">
     <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0000"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0000"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -257,8 +298,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}" name="Table1" displayName="Table1" ref="A1:Q4" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
-  <autoFilter ref="A1:Q4" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}" name="Table1" displayName="Table1" ref="A1:Q7" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+  <autoFilter ref="A1:Q7" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{AECD2685-7611-477D-BB06-D6903AF84BE6}" name="experiment_id" dataDxfId="16"/>
     <tableColumn id="3" xr3:uid="{16EA5037-8320-413B-A37B-8D8E33F69E3F}" name="architecture" dataDxfId="15"/>
@@ -266,17 +307,17 @@
     <tableColumn id="5" xr3:uid="{55257896-9D82-473A-A560-298033D12ADE}" name="epochs_run" dataDxfId="13"/>
     <tableColumn id="17" xr3:uid="{97228026-54D0-4171-A86D-AF6DEA67CC1B}" name="best_epoch" dataDxfId="12"/>
     <tableColumn id="16" xr3:uid="{7E11CAB9-6285-402C-A0BF-68FB93AF36A3}" name="best_val_loss" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{957B48B6-023B-4F02-BCFD-71D690211E27}" name="loss_function" dataDxfId="0"/>
-    <tableColumn id="15" xr3:uid="{107CEEC6-13CB-45B5-A3DD-0F3F173E4C46}" name="optimizer" dataDxfId="10"/>
-    <tableColumn id="14" xr3:uid="{593A2ED1-5C62-4524-B1FC-97F698EED537}" name="lr" dataDxfId="9"/>
-    <tableColumn id="13" xr3:uid="{DEE5E71E-CAFE-4C17-B530-C0735663BA1F}" name="activation_function" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{BFAF2BDA-8ABA-497A-B962-CCB28CC5DE8D}" name="mae" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{0B8CBDEB-5A7B-4A9A-BB91-7AC23A9350D5}" name="mse" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{102009EE-7DD9-45D2-A29C-4A0BE21D4AB9}" name="rmse" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{5282C0F6-8584-43B2-8846-199B2C706B0D}" name="r2" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{23610184-09F0-4909-9C6D-E7DECFEF5B72}" name="mape" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{2E6E547C-B286-4837-8C73-9B2FE1B19668}" name="observation" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{853F7192-7A8A-43FD-BE88-378A3805100E}" name="result" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{957B48B6-023B-4F02-BCFD-71D690211E27}" name="loss_function" dataDxfId="10"/>
+    <tableColumn id="15" xr3:uid="{107CEEC6-13CB-45B5-A3DD-0F3F173E4C46}" name="optimizer" dataDxfId="9"/>
+    <tableColumn id="14" xr3:uid="{593A2ED1-5C62-4524-B1FC-97F698EED537}" name="lr" dataDxfId="8"/>
+    <tableColumn id="13" xr3:uid="{DEE5E71E-CAFE-4C17-B530-C0735663BA1F}" name="activation_function" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{BFAF2BDA-8ABA-497A-B962-CCB28CC5DE8D}" name="mae" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{0B8CBDEB-5A7B-4A9A-BB91-7AC23A9350D5}" name="mse" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{102009EE-7DD9-45D2-A29C-4A0BE21D4AB9}" name="rmse" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{5282C0F6-8584-43B2-8846-199B2C706B0D}" name="r2" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{23610184-09F0-4909-9C6D-E7DECFEF5B72}" name="mape" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{2E6E547C-B286-4837-8C73-9B2FE1B19668}" name="observation" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{853F7192-7A8A-43FD-BE88-378A3805100E}" name="result" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -545,23 +586,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="9.5703125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="9.5703125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="32.85546875" style="2" customWidth="1"/>
+    <col min="4" max="5" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="15.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="32" style="2" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="23.42578125" style="1" customWidth="1"/>
     <col min="18" max="16384" width="9.140625" style="1"/>
   </cols>
@@ -650,19 +691,19 @@
       <c r="J2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="3">
         <v>4998.0600000000004</v>
       </c>
-      <c r="L2" s="1">
+      <c r="L2" s="3">
         <v>40831695.520000003</v>
       </c>
-      <c r="M2" s="1">
+      <c r="M2" s="3">
         <v>6389.97</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="4">
         <v>0.79530000000000001</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="4">
         <v>8.4900000000000003E-2</v>
       </c>
       <c r="P2" s="2" t="s">
@@ -703,19 +744,19 @@
       <c r="J3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="3">
         <v>4747.76</v>
       </c>
-      <c r="L3" s="1">
+      <c r="L3" s="3">
         <v>42827911.909999996</v>
       </c>
-      <c r="M3" s="1">
+      <c r="M3" s="3">
         <v>6544.3</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="4">
         <v>0.7853</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="4">
         <v>7.4300000000000005E-2</v>
       </c>
       <c r="P3" s="2" t="s">
@@ -756,19 +797,19 @@
       <c r="J4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="3">
         <v>5341.39</v>
       </c>
-      <c r="L4" s="1">
+      <c r="L4" s="3">
         <v>50073269.460000001</v>
       </c>
-      <c r="M4" s="1">
+      <c r="M4" s="3">
         <v>7076.25</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="4">
         <v>0.749</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="4">
         <v>8.6699999999999999E-2</v>
       </c>
       <c r="P4" s="2" t="s">
@@ -776,6 +817,165 @@
       </c>
       <c r="Q4" s="2" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="1">
+        <v>144</v>
+      </c>
+      <c r="D5" s="1">
+        <v>17</v>
+      </c>
+      <c r="E5" s="1">
+        <v>10</v>
+      </c>
+      <c r="F5" s="1">
+        <v>3.3660000000000002E-2</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K5" s="3">
+        <v>5705.36</v>
+      </c>
+      <c r="L5" s="3">
+        <v>54950152.119999997</v>
+      </c>
+      <c r="M5" s="3">
+        <v>7412.84</v>
+      </c>
+      <c r="N5" s="4">
+        <v>0.72450000000000003</v>
+      </c>
+      <c r="O5" s="4">
+        <v>9.7699999999999995E-2</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q5" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="1">
+        <v>144</v>
+      </c>
+      <c r="D6" s="1">
+        <v>3</v>
+      </c>
+      <c r="E6" s="1">
+        <v>10</v>
+      </c>
+      <c r="F6" s="1">
+        <v>5.8400000000000001E-2</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K6" s="3">
+        <v>7589.35</v>
+      </c>
+      <c r="L6" s="3">
+        <v>80059016.599999994</v>
+      </c>
+      <c r="M6" s="3">
+        <v>8947.57</v>
+      </c>
+      <c r="N6" s="4">
+        <v>0.59860000000000002</v>
+      </c>
+      <c r="O6" s="4">
+        <v>0.1278</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="1">
+        <v>36</v>
+      </c>
+      <c r="D7" s="1">
+        <v>20</v>
+      </c>
+      <c r="E7" s="1">
+        <v>13</v>
+      </c>
+      <c r="F7" s="1">
+        <v>7.639E-2</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K7" s="3">
+        <v>4979</v>
+      </c>
+      <c r="L7" s="3">
+        <v>50833638.710000001</v>
+      </c>
+      <c r="M7" s="3">
+        <v>7129.77</v>
+      </c>
+      <c r="N7" s="4">
+        <v>0.74509999999999998</v>
+      </c>
+      <c r="O7" s="4">
+        <v>7.1199999999999999E-2</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q7" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: tested more LSTM architectures
</commit_message>
<xml_diff>
--- a/data/experiment_logs.xlsx
+++ b/data/experiment_logs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saadm\Documents\gridops-ai\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62B8A190-E425-4C2C-94C7-106D0BB97E84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66A4C95D-9BE9-40A6-8B01-7D59BBA86506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="52">
   <si>
     <t>experiment_id</t>
   </si>
@@ -159,6 +159,39 @@
   </si>
   <si>
     <t>Not selected; short lookback fails to capture long-term seasonal peaks adequately</t>
+  </si>
+  <si>
+    <t>lstm_7</t>
+  </si>
+  <si>
+    <t>32/0.2/16/1</t>
+  </si>
+  <si>
+    <t>lstm_8</t>
+  </si>
+  <si>
+    <t>128/0.2/64/0.2/32/1</t>
+  </si>
+  <si>
+    <t>Complex multi-layer architecture with a short lookback achieves strong convergence and peak capture</t>
+  </si>
+  <si>
+    <t>lstm_9</t>
+  </si>
+  <si>
+    <t>Huber loss has decreased R2 and overall MAPE has gone significatnly high</t>
+  </si>
+  <si>
+    <t>Best LSTM result so far; retain for comparison</t>
+  </si>
+  <si>
+    <t>Not selected; worse test metrics than MSE</t>
+  </si>
+  <si>
+    <t>Architecture is too simplistic and performs worse with dropout layer</t>
+  </si>
+  <si>
+    <t>Not selected; consider a complex architecture and peak data perfromance</t>
   </si>
 </sst>
 </file>
@@ -203,7 +236,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -215,6 +248,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -298,8 +334,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}" name="Table1" displayName="Table1" ref="A1:Q7" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
-  <autoFilter ref="A1:Q7" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}" name="Table1" displayName="Table1" ref="A1:Q11" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+  <autoFilter ref="A1:Q11" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{AECD2685-7611-477D-BB06-D6903AF84BE6}" name="experiment_id" dataDxfId="16"/>
     <tableColumn id="3" xr3:uid="{16EA5037-8320-413B-A37B-8D8E33F69E3F}" name="architecture" dataDxfId="15"/>
@@ -586,11 +622,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="15.140625" style="1" bestFit="1" customWidth="1"/>
@@ -599,7 +635,7 @@
     <col min="10" max="10" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9" style="4" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="7" style="4" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="8.42578125" style="4" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="32" style="2" bestFit="1" customWidth="1"/>
@@ -883,10 +919,10 @@
         <v>144</v>
       </c>
       <c r="D6" s="1">
+        <v>10</v>
+      </c>
+      <c r="E6" s="1">
         <v>3</v>
-      </c>
-      <c r="E6" s="1">
-        <v>10</v>
       </c>
       <c r="F6" s="1">
         <v>5.8400000000000001E-2</v>
@@ -977,6 +1013,171 @@
       <c r="Q7" s="2" t="s">
         <v>40</v>
       </c>
+    </row>
+    <row r="8" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="1">
+        <v>36</v>
+      </c>
+      <c r="D8" s="1">
+        <v>16</v>
+      </c>
+      <c r="E8" s="1">
+        <v>9</v>
+      </c>
+      <c r="F8" s="1">
+        <v>7.7560000000000004E-2</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K8" s="3">
+        <v>6072.95</v>
+      </c>
+      <c r="L8" s="3">
+        <v>64652855.229999997</v>
+      </c>
+      <c r="M8" s="3">
+        <v>8040.7</v>
+      </c>
+      <c r="N8" s="4">
+        <v>0.67589999999999995</v>
+      </c>
+      <c r="O8" s="4">
+        <v>0.1009</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="1">
+        <v>36</v>
+      </c>
+      <c r="D9" s="1">
+        <v>32</v>
+      </c>
+      <c r="E9" s="1">
+        <v>25</v>
+      </c>
+      <c r="F9" s="1">
+        <v>4.4209999999999999E-2</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K9" s="3">
+        <v>4153.9399999999996</v>
+      </c>
+      <c r="L9" s="3">
+        <v>38190945.700000003</v>
+      </c>
+      <c r="M9" s="3">
+        <v>6179.88</v>
+      </c>
+      <c r="N9" s="4">
+        <v>0.8085</v>
+      </c>
+      <c r="O9" s="5">
+        <v>6.5500000000000003E-2</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="1">
+        <v>36</v>
+      </c>
+      <c r="D10" s="1">
+        <v>22</v>
+      </c>
+      <c r="E10" s="1">
+        <v>15</v>
+      </c>
+      <c r="F10" s="1">
+        <v>2.121E-2</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K10" s="3">
+        <v>5874.28</v>
+      </c>
+      <c r="L10" s="3">
+        <v>65417803.210000001</v>
+      </c>
+      <c r="M10" s="3">
+        <v>8088.13</v>
+      </c>
+      <c r="N10" s="4">
+        <v>0.67200000000000004</v>
+      </c>
+      <c r="O10" s="4">
+        <v>0.1027</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q10" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="Q11" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
feat: added 2 new plots to compare LSTM and Seasonal Naive predictions with actual demand
</commit_message>
<xml_diff>
--- a/data/experiment_logs.xlsx
+++ b/data/experiment_logs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saadm\Documents\gridops-ai\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66A4C95D-9BE9-40A6-8B01-7D59BBA86506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC025F0-53F7-44AD-A400-F006E5AAA7F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -625,21 +625,22 @@
   <dimension ref="A1:Q11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="15.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="32" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="23.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="19" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="52" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="30.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="18" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
feat: Improved LSTM performance with seasonal lag feature reflecting seasonal naive performance.
</commit_message>
<xml_diff>
--- a/data/experiment_logs.xlsx
+++ b/data/experiment_logs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saadm\Documents\gridops-ai\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC025F0-53F7-44AD-A400-F006E5AAA7F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7CFF033-CC51-4135-8EA5-3C8770727C75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="59">
   <si>
     <t>experiment_id</t>
   </si>
@@ -192,6 +192,27 @@
   </si>
   <si>
     <t>Not selected; consider a complex architecture and peak data perfromance</t>
+  </si>
+  <si>
+    <t>lstm_10</t>
+  </si>
+  <si>
+    <t>batch_size</t>
+  </si>
+  <si>
+    <t>Performance improved; train with smaller batches</t>
+  </si>
+  <si>
+    <t>With the addition of 138 timestep lag feature, as being used in Seasonal Naïve model, LSTM performance improved</t>
+  </si>
+  <si>
+    <t>lstm_11</t>
+  </si>
+  <si>
+    <t>Based on the plots, peak performance dropped with change in batch size but resudual mean moved closer to 0</t>
+  </si>
+  <si>
+    <t>Train with a longer lookback as a trail</t>
   </si>
 </sst>
 </file>
@@ -257,7 +278,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="20">
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -334,26 +358,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}" name="Table1" displayName="Table1" ref="A1:Q11" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
-  <autoFilter ref="A1:Q11" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}"/>
-  <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{AECD2685-7611-477D-BB06-D6903AF84BE6}" name="experiment_id" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{16EA5037-8320-413B-A37B-8D8E33F69E3F}" name="architecture" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{BDD197F5-ADC5-4496-A783-AF42D3213569}" name="lookback" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{55257896-9D82-473A-A560-298033D12ADE}" name="epochs_run" dataDxfId="13"/>
-    <tableColumn id="17" xr3:uid="{97228026-54D0-4171-A86D-AF6DEA67CC1B}" name="best_epoch" dataDxfId="12"/>
-    <tableColumn id="16" xr3:uid="{7E11CAB9-6285-402C-A0BF-68FB93AF36A3}" name="best_val_loss" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{957B48B6-023B-4F02-BCFD-71D690211E27}" name="loss_function" dataDxfId="10"/>
-    <tableColumn id="15" xr3:uid="{107CEEC6-13CB-45B5-A3DD-0F3F173E4C46}" name="optimizer" dataDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{593A2ED1-5C62-4524-B1FC-97F698EED537}" name="lr" dataDxfId="8"/>
-    <tableColumn id="13" xr3:uid="{DEE5E71E-CAFE-4C17-B530-C0735663BA1F}" name="activation_function" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{BFAF2BDA-8ABA-497A-B962-CCB28CC5DE8D}" name="mae" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{0B8CBDEB-5A7B-4A9A-BB91-7AC23A9350D5}" name="mse" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{102009EE-7DD9-45D2-A29C-4A0BE21D4AB9}" name="rmse" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{5282C0F6-8584-43B2-8846-199B2C706B0D}" name="r2" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{23610184-09F0-4909-9C6D-E7DECFEF5B72}" name="mape" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{2E6E547C-B286-4837-8C73-9B2FE1B19668}" name="observation" dataDxfId="1"/>
-    <tableColumn id="12" xr3:uid="{853F7192-7A8A-43FD-BE88-378A3805100E}" name="result" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}" name="Table1" displayName="Table1" ref="A1:R12" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+  <autoFilter ref="A1:R12" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}"/>
+  <tableColumns count="18">
+    <tableColumn id="1" xr3:uid="{AECD2685-7611-477D-BB06-D6903AF84BE6}" name="experiment_id" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{16EA5037-8320-413B-A37B-8D8E33F69E3F}" name="architecture" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{BDD197F5-ADC5-4496-A783-AF42D3213569}" name="lookback" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{55257896-9D82-473A-A560-298033D12ADE}" name="epochs_run" dataDxfId="14"/>
+    <tableColumn id="17" xr3:uid="{97228026-54D0-4171-A86D-AF6DEA67CC1B}" name="best_epoch" dataDxfId="13"/>
+    <tableColumn id="16" xr3:uid="{7E11CAB9-6285-402C-A0BF-68FB93AF36A3}" name="best_val_loss" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{957B48B6-023B-4F02-BCFD-71D690211E27}" name="loss_function" dataDxfId="11"/>
+    <tableColumn id="15" xr3:uid="{107CEEC6-13CB-45B5-A3DD-0F3F173E4C46}" name="optimizer" dataDxfId="10"/>
+    <tableColumn id="14" xr3:uid="{593A2ED1-5C62-4524-B1FC-97F698EED537}" name="lr" dataDxfId="9"/>
+    <tableColumn id="18" xr3:uid="{CEE0339B-8441-4C51-BACE-44E6312D5E25}" name="batch_size" dataDxfId="0"/>
+    <tableColumn id="13" xr3:uid="{DEE5E71E-CAFE-4C17-B530-C0735663BA1F}" name="activation_function" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{BFAF2BDA-8ABA-497A-B962-CCB28CC5DE8D}" name="mae" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{0B8CBDEB-5A7B-4A9A-BB91-7AC23A9350D5}" name="mse" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{102009EE-7DD9-45D2-A29C-4A0BE21D4AB9}" name="rmse" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{5282C0F6-8584-43B2-8846-199B2C706B0D}" name="r2" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{23610184-09F0-4909-9C6D-E7DECFEF5B72}" name="mape" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{2E6E547C-B286-4837-8C73-9B2FE1B19668}" name="observation" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{853F7192-7A8A-43FD-BE88-378A3805100E}" name="result" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -622,10 +647,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="19" style="1" bestFit="1" customWidth="1"/>
@@ -633,18 +658,19 @@
     <col min="7" max="7" width="21.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="28.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="52" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="30.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="1"/>
+    <col min="10" max="10" width="18" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="28.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="45.5703125" style="2" customWidth="1"/>
+    <col min="18" max="18" width="45.28515625" style="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -673,31 +699,34 @@
         <v>14</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -725,32 +754,35 @@
       <c r="I2" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="1">
+        <v>64</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="3">
+      <c r="L2" s="3">
         <v>4998.0600000000004</v>
       </c>
-      <c r="L2" s="3">
+      <c r="M2" s="3">
         <v>40831695.520000003</v>
       </c>
-      <c r="M2" s="3">
+      <c r="N2" s="3">
         <v>6389.97</v>
       </c>
-      <c r="N2" s="4">
+      <c r="O2" s="4">
         <v>0.79530000000000001</v>
       </c>
-      <c r="O2" s="4">
+      <c r="P2" s="4">
         <v>8.4900000000000003E-2</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="Q2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="R2" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
@@ -778,32 +810,35 @@
       <c r="I3" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="1">
+        <v>64</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K3" s="3">
+      <c r="L3" s="3">
         <v>4747.76</v>
       </c>
-      <c r="L3" s="3">
+      <c r="M3" s="3">
         <v>42827911.909999996</v>
       </c>
-      <c r="M3" s="3">
+      <c r="N3" s="3">
         <v>6544.3</v>
       </c>
-      <c r="N3" s="4">
+      <c r="O3" s="4">
         <v>0.7853</v>
       </c>
-      <c r="O3" s="4">
+      <c r="P3" s="4">
         <v>7.4300000000000005E-2</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="R3" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>25</v>
       </c>
@@ -831,32 +866,35 @@
       <c r="I4" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" s="1">
+        <v>64</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K4" s="3">
+      <c r="L4" s="3">
         <v>5341.39</v>
       </c>
-      <c r="L4" s="3">
+      <c r="M4" s="3">
         <v>50073269.460000001</v>
       </c>
-      <c r="M4" s="3">
+      <c r="N4" s="3">
         <v>7076.25</v>
       </c>
-      <c r="N4" s="4">
+      <c r="O4" s="4">
         <v>0.749</v>
       </c>
-      <c r="O4" s="4">
+      <c r="P4" s="4">
         <v>8.6699999999999999E-2</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="Q4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="R4" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>32</v>
       </c>
@@ -884,32 +922,35 @@
       <c r="I5" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="1">
+        <v>64</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="3">
+      <c r="L5" s="3">
         <v>5705.36</v>
       </c>
-      <c r="L5" s="3">
+      <c r="M5" s="3">
         <v>54950152.119999997</v>
       </c>
-      <c r="M5" s="3">
+      <c r="N5" s="3">
         <v>7412.84</v>
       </c>
-      <c r="N5" s="4">
+      <c r="O5" s="4">
         <v>0.72450000000000003</v>
       </c>
-      <c r="O5" s="4">
+      <c r="P5" s="4">
         <v>9.7699999999999995E-2</v>
       </c>
-      <c r="P5" s="2" t="s">
+      <c r="Q5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="Q5" s="2" t="s">
+      <c r="R5" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>33</v>
       </c>
@@ -937,32 +978,35 @@
       <c r="I6" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="1">
+        <v>64</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K6" s="3">
+      <c r="L6" s="3">
         <v>7589.35</v>
       </c>
-      <c r="L6" s="3">
+      <c r="M6" s="3">
         <v>80059016.599999994</v>
       </c>
-      <c r="M6" s="3">
+      <c r="N6" s="3">
         <v>8947.57</v>
       </c>
-      <c r="N6" s="4">
+      <c r="O6" s="4">
         <v>0.59860000000000002</v>
       </c>
-      <c r="O6" s="4">
+      <c r="P6" s="4">
         <v>0.1278</v>
       </c>
-      <c r="P6" s="2" t="s">
+      <c r="Q6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="Q6" s="2" t="s">
+      <c r="R6" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>34</v>
       </c>
@@ -990,32 +1034,35 @@
       <c r="I7" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" s="1">
+        <v>64</v>
+      </c>
+      <c r="K7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K7" s="3">
+      <c r="L7" s="3">
         <v>4979</v>
       </c>
-      <c r="L7" s="3">
+      <c r="M7" s="3">
         <v>50833638.710000001</v>
       </c>
-      <c r="M7" s="3">
+      <c r="N7" s="3">
         <v>7129.77</v>
       </c>
-      <c r="N7" s="4">
+      <c r="O7" s="4">
         <v>0.74509999999999998</v>
       </c>
-      <c r="O7" s="4">
+      <c r="P7" s="4">
         <v>7.1199999999999999E-2</v>
       </c>
-      <c r="P7" s="2" t="s">
+      <c r="Q7" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="Q7" s="2" t="s">
+      <c r="R7" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>41</v>
       </c>
@@ -1043,32 +1090,35 @@
       <c r="I8" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="1">
+        <v>64</v>
+      </c>
+      <c r="K8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K8" s="3">
+      <c r="L8" s="3">
         <v>6072.95</v>
       </c>
-      <c r="L8" s="3">
+      <c r="M8" s="3">
         <v>64652855.229999997</v>
       </c>
-      <c r="M8" s="3">
+      <c r="N8" s="3">
         <v>8040.7</v>
       </c>
-      <c r="N8" s="4">
+      <c r="O8" s="4">
         <v>0.67589999999999995</v>
       </c>
-      <c r="O8" s="4">
+      <c r="P8" s="4">
         <v>0.1009</v>
       </c>
-      <c r="P8" s="2" t="s">
+      <c r="Q8" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="Q8" s="2" t="s">
+      <c r="R8" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>43</v>
       </c>
@@ -1096,32 +1146,35 @@
       <c r="I9" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" s="1">
+        <v>64</v>
+      </c>
+      <c r="K9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K9" s="3">
+      <c r="L9" s="3">
         <v>4153.9399999999996</v>
       </c>
-      <c r="L9" s="3">
+      <c r="M9" s="3">
         <v>38190945.700000003</v>
       </c>
-      <c r="M9" s="3">
+      <c r="N9" s="3">
         <v>6179.88</v>
       </c>
-      <c r="N9" s="4">
+      <c r="O9" s="4">
         <v>0.8085</v>
       </c>
-      <c r="O9" s="5">
+      <c r="P9" s="5">
         <v>6.5500000000000003E-2</v>
       </c>
-      <c r="P9" s="2" t="s">
+      <c r="Q9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="Q9" s="2" t="s">
+      <c r="R9" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>46</v>
       </c>
@@ -1149,36 +1202,145 @@
       <c r="I10" s="1">
         <v>1E-3</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" s="1">
+        <v>64</v>
+      </c>
+      <c r="K10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K10" s="3">
+      <c r="L10" s="3">
         <v>5874.28</v>
       </c>
-      <c r="L10" s="3">
+      <c r="M10" s="3">
         <v>65417803.210000001</v>
       </c>
-      <c r="M10" s="3">
+      <c r="N10" s="3">
         <v>8088.13</v>
       </c>
-      <c r="N10" s="4">
+      <c r="O10" s="4">
         <v>0.67200000000000004</v>
       </c>
-      <c r="O10" s="4">
+      <c r="P10" s="4">
         <v>0.1027</v>
       </c>
-      <c r="P10" s="2" t="s">
+      <c r="Q10" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="Q10" s="2" t="s">
+      <c r="R10" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="Q11" s="2"/>
+    <row r="11" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="1">
+        <v>36</v>
+      </c>
+      <c r="D11" s="1">
+        <v>35</v>
+      </c>
+      <c r="E11" s="1">
+        <v>28</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1.391E-2</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="J11" s="1">
+        <v>64</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="L11" s="3">
+        <v>3768.86</v>
+      </c>
+      <c r="M11" s="3">
+        <v>22150121.68</v>
+      </c>
+      <c r="N11" s="3">
+        <v>4706.3900000000003</v>
+      </c>
+      <c r="O11" s="4">
+        <v>0.88890000000000002</v>
+      </c>
+      <c r="P11" s="5">
+        <v>6.2899999999999998E-2</v>
+      </c>
+      <c r="Q11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="R11" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="1">
+        <v>36</v>
+      </c>
+      <c r="D12" s="1">
+        <v>15</v>
+      </c>
+      <c r="E12" s="1">
+        <v>8</v>
+      </c>
+      <c r="F12" s="1">
+        <v>4.2999999999999997E-2</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I12" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="J12" s="1">
+        <v>32</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="L12" s="3">
+        <v>4016.71</v>
+      </c>
+      <c r="M12" s="3">
+        <v>24984631.32</v>
+      </c>
+      <c r="N12" s="3">
+        <v>4998.46</v>
+      </c>
+      <c r="O12" s="4">
+        <v>0.87470000000000003</v>
+      </c>
+      <c r="P12" s="4">
+        <v>6.6400000000000001E-2</v>
+      </c>
+      <c r="Q12" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="R12" s="2" t="s">
+        <v>58</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
feat: updated with more LSTM training.
</commit_message>
<xml_diff>
--- a/data/experiment_logs.xlsx
+++ b/data/experiment_logs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saadm\Documents\gridops-ai\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7CFF033-CC51-4135-8EA5-3C8770727C75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F37EFEE6-422C-4B8B-AD47-8C8F30F9FCC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="62">
   <si>
     <t>experiment_id</t>
   </si>
@@ -213,6 +213,15 @@
   </si>
   <si>
     <t>Train with a longer lookback as a trail</t>
+  </si>
+  <si>
+    <t>lstm_12</t>
+  </si>
+  <si>
+    <t>A longer lookback window with new feature performed best. LSTM peak period MAE is still worse than seasonal naïve</t>
+  </si>
+  <si>
+    <t>Training resulted in a better model as the plots reflect</t>
   </si>
 </sst>
 </file>
@@ -237,12 +246,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -257,7 +272,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -274,15 +289,24 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="20">
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -310,6 +334,9 @@
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -358,8 +385,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}" name="Table1" displayName="Table1" ref="A1:R12" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
-  <autoFilter ref="A1:R12" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}" name="Table1" displayName="Table1" ref="A1:R13" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+  <autoFilter ref="A1:R13" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}"/>
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{AECD2685-7611-477D-BB06-D6903AF84BE6}" name="experiment_id" dataDxfId="17"/>
     <tableColumn id="3" xr3:uid="{16EA5037-8320-413B-A37B-8D8E33F69E3F}" name="architecture" dataDxfId="16"/>
@@ -370,15 +397,15 @@
     <tableColumn id="2" xr3:uid="{957B48B6-023B-4F02-BCFD-71D690211E27}" name="loss_function" dataDxfId="11"/>
     <tableColumn id="15" xr3:uid="{107CEEC6-13CB-45B5-A3DD-0F3F173E4C46}" name="optimizer" dataDxfId="10"/>
     <tableColumn id="14" xr3:uid="{593A2ED1-5C62-4524-B1FC-97F698EED537}" name="lr" dataDxfId="9"/>
-    <tableColumn id="18" xr3:uid="{CEE0339B-8441-4C51-BACE-44E6312D5E25}" name="batch_size" dataDxfId="0"/>
-    <tableColumn id="13" xr3:uid="{DEE5E71E-CAFE-4C17-B530-C0735663BA1F}" name="activation_function" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{BFAF2BDA-8ABA-497A-B962-CCB28CC5DE8D}" name="mae" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{0B8CBDEB-5A7B-4A9A-BB91-7AC23A9350D5}" name="mse" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{102009EE-7DD9-45D2-A29C-4A0BE21D4AB9}" name="rmse" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{5282C0F6-8584-43B2-8846-199B2C706B0D}" name="r2" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{23610184-09F0-4909-9C6D-E7DECFEF5B72}" name="mape" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{2E6E547C-B286-4837-8C73-9B2FE1B19668}" name="observation" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{853F7192-7A8A-43FD-BE88-378A3805100E}" name="result" dataDxfId="1"/>
+    <tableColumn id="18" xr3:uid="{CEE0339B-8441-4C51-BACE-44E6312D5E25}" name="batch_size" dataDxfId="8"/>
+    <tableColumn id="13" xr3:uid="{DEE5E71E-CAFE-4C17-B530-C0735663BA1F}" name="activation_function" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{BFAF2BDA-8ABA-497A-B962-CCB28CC5DE8D}" name="mae" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{0B8CBDEB-5A7B-4A9A-BB91-7AC23A9350D5}" name="mse" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{102009EE-7DD9-45D2-A29C-4A0BE21D4AB9}" name="rmse" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{5282C0F6-8584-43B2-8846-199B2C706B0D}" name="r2" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{23610184-09F0-4909-9C6D-E7DECFEF5B72}" name="mape" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{2E6E547C-B286-4837-8C73-9B2FE1B19668}" name="observation" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{853F7192-7A8A-43FD-BE88-378A3805100E}" name="result" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -647,7 +674,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R12"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" style="1" customWidth="1"/>
@@ -1342,6 +1369,62 @@
         <v>58</v>
       </c>
     </row>
+    <row r="13" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="6">
+        <v>144</v>
+      </c>
+      <c r="D13" s="6">
+        <v>24</v>
+      </c>
+      <c r="E13" s="6">
+        <v>17</v>
+      </c>
+      <c r="F13" s="6">
+        <v>1.421E-2</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I13" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="J13" s="6">
+        <v>32</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L13" s="7">
+        <v>3178.43</v>
+      </c>
+      <c r="M13" s="7">
+        <v>16154198.52</v>
+      </c>
+      <c r="N13" s="7">
+        <v>4019.23</v>
+      </c>
+      <c r="O13" s="8">
+        <v>0.91900000000000004</v>
+      </c>
+      <c r="P13" s="8">
+        <v>5.5399999999999998E-2</v>
+      </c>
+      <c r="Q13" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="R13" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: final testing results of LSTM updated
</commit_message>
<xml_diff>
--- a/data/experiment_logs.xlsx
+++ b/data/experiment_logs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saadm\Documents\gridops-ai\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F37EFEE6-422C-4B8B-AD47-8C8F30F9FCC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92ECA422-4413-4007-82CE-62AD948D8C0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="65">
   <si>
     <t>experiment_id</t>
   </si>
@@ -222,6 +222,15 @@
   </si>
   <si>
     <t>Training resulted in a better model as the plots reflect</t>
+  </si>
+  <si>
+    <t>lstm_13</t>
+  </si>
+  <si>
+    <t>Adding cyclical time as features improved the model significantly. Peak period performance has not improved much</t>
+  </si>
+  <si>
+    <t>Best model. Finalised.</t>
   </si>
 </sst>
 </file>
@@ -272,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -301,6 +310,18 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -385,8 +406,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}" name="Table1" displayName="Table1" ref="A1:R13" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
-  <autoFilter ref="A1:R13" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}" name="Table1" displayName="Table1" ref="A1:R14" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+  <autoFilter ref="A1:R14" xr:uid="{ED8F316B-B602-48FE-8745-23276654EA86}"/>
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{AECD2685-7611-477D-BB06-D6903AF84BE6}" name="experiment_id" dataDxfId="17"/>
     <tableColumn id="3" xr3:uid="{16EA5037-8320-413B-A37B-8D8E33F69E3F}" name="architecture" dataDxfId="16"/>
@@ -674,7 +695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" style="1" customWidth="1"/>
@@ -1370,59 +1391,115 @@
       </c>
     </row>
     <row r="13" spans="1:18" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="10">
         <v>144</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="10">
         <v>24</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="10">
         <v>17</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="10">
         <v>1.421E-2</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="H13" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="6">
+      <c r="I13" s="10">
         <v>1E-3</v>
       </c>
-      <c r="J13" s="6">
+      <c r="J13" s="10">
         <v>32</v>
       </c>
-      <c r="K13" s="6" t="s">
+      <c r="K13" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="L13" s="7">
+      <c r="L13" s="11">
         <v>3178.43</v>
       </c>
-      <c r="M13" s="7">
+      <c r="M13" s="11">
         <v>16154198.52</v>
       </c>
-      <c r="N13" s="7">
+      <c r="N13" s="11">
         <v>4019.23</v>
       </c>
-      <c r="O13" s="8">
+      <c r="O13" s="12">
         <v>0.91900000000000004</v>
       </c>
-      <c r="P13" s="8">
+      <c r="P13" s="12">
         <v>5.5399999999999998E-2</v>
       </c>
-      <c r="Q13" s="9" t="s">
+      <c r="Q13" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="R13" s="9" t="s">
+      <c r="R13" s="13" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="6">
+        <v>144</v>
+      </c>
+      <c r="D14" s="6">
+        <v>35</v>
+      </c>
+      <c r="E14" s="6">
+        <v>28</v>
+      </c>
+      <c r="F14" s="6">
+        <v>1.106E-2</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I14" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="J14" s="6">
+        <v>32</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L14" s="7">
+        <v>2798.4</v>
+      </c>
+      <c r="M14" s="7">
+        <v>12345560.369999999</v>
+      </c>
+      <c r="N14" s="7">
+        <v>3513.62</v>
+      </c>
+      <c r="O14" s="8">
+        <v>0.93810000000000004</v>
+      </c>
+      <c r="P14" s="8">
+        <v>4.53E-2</v>
+      </c>
+      <c r="Q14" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="R14" s="9" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>